<commit_message>
Update Dexcom job tracker
</commit_message>
<xml_diff>
--- a/Dexcom_Job_Tracker.xlsx
+++ b/Dexcom_Job_Tracker.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Dexcom Job Tracker" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Dexcom Job Tracker'!$A$1:$D$63</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Dexcom Job Tracker'!$A$1:$D$65</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -84,7 +84,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -95,6 +95,15 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
@@ -482,7 +491,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D63"/>
+  <dimension ref="A1:D65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1753,8 +1762,48 @@
         </is>
       </c>
     </row>
+    <row r="64">
+      <c r="A64" s="12" t="inlineStr">
+        <is>
+          <t>Singapore</t>
+        </is>
+      </c>
+      <c r="B64" s="13" t="n">
+        <v>46268</v>
+      </c>
+      <c r="C64" s="4" t="inlineStr">
+        <is>
+          <t>APAC FP&amp;A Manager</t>
+        </is>
+      </c>
+      <c r="D64" s="14" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/view/4462770899/</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="12" t="inlineStr">
+        <is>
+          <t>Spain</t>
+        </is>
+      </c>
+      <c r="B65" s="13" t="n">
+        <v>46268</v>
+      </c>
+      <c r="C65" s="4" t="inlineStr">
+        <is>
+          <t>Commercial Analytics &amp; Operations Associate</t>
+        </is>
+      </c>
+      <c r="D65" s="14" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/view/4462778751/</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:D63"/>
+  <autoFilter ref="A1:D65"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D3" r:id="rId2"/>
@@ -1818,6 +1867,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D61" r:id="rId60"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D62" r:id="rId61"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D63" r:id="rId62"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D64" r:id="rId63"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D65" r:id="rId64"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>